<commit_message>
feat: add seasonal revenue factor analysis table to overview dashboard and aggregate quarterly values in DT_CTTV_2025.xlsx sheet
</commit_message>
<xml_diff>
--- a/DT_CTTV_2025.xlsx
+++ b/DT_CTTV_2025.xlsx
@@ -7,6 +7,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng doanh thu quý" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$2:$G$322</definedName>
@@ -444,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H322"/>
+  <dimension ref="A2:H322"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9.85546875" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -452,7 +453,6 @@
     <col width="21.42578125" bestFit="1" customWidth="1" style="7" min="3" max="7"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2" customFormat="1" s="6">
       <c r="A2" s="4" t="inlineStr">
         <is>
@@ -10739,4 +10739,1565 @@
   <autoFilter ref="A2:G322"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E81"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Tên đơn vị</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Quý 1</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Quý 2</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Quý 3</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Quý 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>BV An Giang</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>24850697840</v>
+      </c>
+      <c r="C2" t="n">
+        <v>10814853829</v>
+      </c>
+      <c r="D2" t="n">
+        <v>45494049538</v>
+      </c>
+      <c r="E2" t="n">
+        <v>23100156172</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>BV An Phú</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>25812053170</v>
+      </c>
+      <c r="C3" t="n">
+        <v>23336299000</v>
+      </c>
+      <c r="D3" t="n">
+        <v>19669456456</v>
+      </c>
+      <c r="E3" t="n">
+        <v>26437426635</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>BV Bà Rịa - Vũng Tàu</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>20470818929</v>
+      </c>
+      <c r="C4" t="n">
+        <v>7274463333</v>
+      </c>
+      <c r="D4" t="n">
+        <v>6457720848</v>
+      </c>
+      <c r="E4" t="n">
+        <v>5533348352</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>BV Bình Dương</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>14419502142</v>
+      </c>
+      <c r="C5" t="n">
+        <v>18275624386</v>
+      </c>
+      <c r="D5" t="n">
+        <v>22804235074</v>
+      </c>
+      <c r="E5" t="n">
+        <v>26682280009</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>BV Bình Phước</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>8139485842</v>
+      </c>
+      <c r="C6" t="n">
+        <v>7118985669</v>
+      </c>
+      <c r="D6" t="n">
+        <v>8019093993</v>
+      </c>
+      <c r="E6" t="n">
+        <v>11524422522</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>BV Bình Thuận</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>15003817039</v>
+      </c>
+      <c r="C7" t="n">
+        <v>13054624918</v>
+      </c>
+      <c r="D7" t="n">
+        <v>49425313067</v>
+      </c>
+      <c r="E7" t="n">
+        <v>18525018454</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>BV Bình Định</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>12620839402</v>
+      </c>
+      <c r="C8" t="n">
+        <v>12398509407</v>
+      </c>
+      <c r="D8" t="n">
+        <v>13153719791</v>
+      </c>
+      <c r="E8" t="n">
+        <v>16916989262</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>BV Bạc Liêu</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>4473451571</v>
+      </c>
+      <c r="C9" t="n">
+        <v>4334403713</v>
+      </c>
+      <c r="D9" t="n">
+        <v>7822239592</v>
+      </c>
+      <c r="E9" t="n">
+        <v>6378916727</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>BV Bắc Cạn</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1573834105</v>
+      </c>
+      <c r="C10" t="n">
+        <v>1329680198</v>
+      </c>
+      <c r="D10" t="n">
+        <v>2116469250</v>
+      </c>
+      <c r="E10" t="n">
+        <v>2236296495</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>BV Bắc Giang</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>12076777969</v>
+      </c>
+      <c r="C11" t="n">
+        <v>17124595702</v>
+      </c>
+      <c r="D11" t="n">
+        <v>16609813654</v>
+      </c>
+      <c r="E11" t="n">
+        <v>28700818127</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>BV Bắc Ninh</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>12031945926</v>
+      </c>
+      <c r="C12" t="n">
+        <v>14304097619</v>
+      </c>
+      <c r="D12" t="n">
+        <v>24168747219</v>
+      </c>
+      <c r="E12" t="n">
+        <v>32260327578</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>BV Bến Thành</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>15115618740</v>
+      </c>
+      <c r="C13" t="n">
+        <v>19296727933</v>
+      </c>
+      <c r="D13" t="n">
+        <v>23681548397</v>
+      </c>
+      <c r="E13" t="n">
+        <v>19220097204</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>BV Bến Tre</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>3225612322</v>
+      </c>
+      <c r="C14" t="n">
+        <v>3710952840</v>
+      </c>
+      <c r="D14" t="n">
+        <v>30734453111</v>
+      </c>
+      <c r="E14" t="n">
+        <v>5245350692</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>BV Cao Bằng</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>3258065494</v>
+      </c>
+      <c r="C15" t="n">
+        <v>3173370672</v>
+      </c>
+      <c r="D15" t="n">
+        <v>2629032420</v>
+      </c>
+      <c r="E15" t="n">
+        <v>3728208002</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>BV Cà Mau</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>4531445986</v>
+      </c>
+      <c r="C16" t="n">
+        <v>6145516488</v>
+      </c>
+      <c r="D16" t="n">
+        <v>5163923724</v>
+      </c>
+      <c r="E16" t="n">
+        <v>6735922491</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>BV Cần Thơ</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>20114592389</v>
+      </c>
+      <c r="C17" t="n">
+        <v>19717049624</v>
+      </c>
+      <c r="D17" t="n">
+        <v>28998004936</v>
+      </c>
+      <c r="E17" t="n">
+        <v>24880497773</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>BV Dak Lak</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>14501039956</v>
+      </c>
+      <c r="C18" t="n">
+        <v>16930197406</v>
+      </c>
+      <c r="D18" t="n">
+        <v>15987675908</v>
+      </c>
+      <c r="E18" t="n">
+        <v>21087875367</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>BV Dak Nong</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>3975272361</v>
+      </c>
+      <c r="C19" t="n">
+        <v>4377468359</v>
+      </c>
+      <c r="D19" t="n">
+        <v>4834747097</v>
+      </c>
+      <c r="E19" t="n">
+        <v>6302001288</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>BV Gia Lai</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>13571066243</v>
+      </c>
+      <c r="C20" t="n">
+        <v>10848206726</v>
+      </c>
+      <c r="D20" t="n">
+        <v>12080217722</v>
+      </c>
+      <c r="E20" t="n">
+        <v>15626047343</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>BV Gia Định</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>15282019468</v>
+      </c>
+      <c r="C21" t="n">
+        <v>17312808726</v>
+      </c>
+      <c r="D21" t="n">
+        <v>14287270118</v>
+      </c>
+      <c r="E21" t="n">
+        <v>17491897638</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>BV Hà Giang</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>4310198573</v>
+      </c>
+      <c r="C22" t="n">
+        <v>4176531016</v>
+      </c>
+      <c r="D22" t="n">
+        <v>3905554372</v>
+      </c>
+      <c r="E22" t="n">
+        <v>5351771365</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>BV Hà Nam</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>4040326499</v>
+      </c>
+      <c r="C23" t="n">
+        <v>6206091747</v>
+      </c>
+      <c r="D23" t="n">
+        <v>7161858706</v>
+      </c>
+      <c r="E23" t="n">
+        <v>7908608249</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>BV Hà Nội</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>85092367322</v>
+      </c>
+      <c r="C24" t="n">
+        <v>77609794241</v>
+      </c>
+      <c r="D24" t="n">
+        <v>70314842919</v>
+      </c>
+      <c r="E24" t="n">
+        <v>97209244613</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>BV Hà Thành</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>86447993781</v>
+      </c>
+      <c r="C25" t="n">
+        <v>53172362584</v>
+      </c>
+      <c r="D25" t="n">
+        <v>55588577676</v>
+      </c>
+      <c r="E25" t="n">
+        <v>51891114060</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>BV Hà Tĩnh</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>8234139729</v>
+      </c>
+      <c r="C26" t="n">
+        <v>9516229053</v>
+      </c>
+      <c r="D26" t="n">
+        <v>12537155853</v>
+      </c>
+      <c r="E26" t="n">
+        <v>15178468769</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>BV Hòa Bình</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>4394179933</v>
+      </c>
+      <c r="C27" t="n">
+        <v>4053581007</v>
+      </c>
+      <c r="D27" t="n">
+        <v>5104337986</v>
+      </c>
+      <c r="E27" t="n">
+        <v>5980213210</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>BV Hưng Yên</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>11116754018</v>
+      </c>
+      <c r="C28" t="n">
+        <v>17018283082</v>
+      </c>
+      <c r="D28" t="n">
+        <v>48698140005</v>
+      </c>
+      <c r="E28" t="n">
+        <v>18418331660</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>BV Hải Dương</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>10584080052</v>
+      </c>
+      <c r="C29" t="n">
+        <v>12347265206</v>
+      </c>
+      <c r="D29" t="n">
+        <v>40640775933</v>
+      </c>
+      <c r="E29" t="n">
+        <v>25578912224</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>BV Hải Phòng</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>16612742209</v>
+      </c>
+      <c r="C30" t="n">
+        <v>19910275752</v>
+      </c>
+      <c r="D30" t="n">
+        <v>25387965781</v>
+      </c>
+      <c r="E30" t="n">
+        <v>29196590419</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>BV Hậu Giang</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>8220042497</v>
+      </c>
+      <c r="C31" t="n">
+        <v>6356149387</v>
+      </c>
+      <c r="D31" t="n">
+        <v>12334352426</v>
+      </c>
+      <c r="E31" t="n">
+        <v>12117043953</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>BV Khánh Hòa</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>19406416153</v>
+      </c>
+      <c r="C32" t="n">
+        <v>15227227741</v>
+      </c>
+      <c r="D32" t="n">
+        <v>18755734034</v>
+      </c>
+      <c r="E32" t="n">
+        <v>20318283978</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>BV Kiên Giang</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>25518368353</v>
+      </c>
+      <c r="C33" t="n">
+        <v>23641322779</v>
+      </c>
+      <c r="D33" t="n">
+        <v>34221229195</v>
+      </c>
+      <c r="E33" t="n">
+        <v>51239504702</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>BV Kon Tum</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>4196146419</v>
+      </c>
+      <c r="C34" t="n">
+        <v>4339728040</v>
+      </c>
+      <c r="D34" t="n">
+        <v>4326906535</v>
+      </c>
+      <c r="E34" t="n">
+        <v>6205652836</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>BV Lai Châu</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>1594772837</v>
+      </c>
+      <c r="C35" t="n">
+        <v>1394003377</v>
+      </c>
+      <c r="D35" t="n">
+        <v>1429084631</v>
+      </c>
+      <c r="E35" t="n">
+        <v>2147190741</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>BV Long An</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>7047948964</v>
+      </c>
+      <c r="C36" t="n">
+        <v>6129567160</v>
+      </c>
+      <c r="D36" t="n">
+        <v>10849932895</v>
+      </c>
+      <c r="E36" t="n">
+        <v>13929165303</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>BV Long Thành</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>5727258885</v>
+      </c>
+      <c r="C37" t="n">
+        <v>4635486066</v>
+      </c>
+      <c r="D37" t="n">
+        <v>6156921972</v>
+      </c>
+      <c r="E37" t="n">
+        <v>16332911136</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>BV Lào Cai</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>3432973287</v>
+      </c>
+      <c r="C38" t="n">
+        <v>3982950223</v>
+      </c>
+      <c r="D38" t="n">
+        <v>4616367836</v>
+      </c>
+      <c r="E38" t="n">
+        <v>4857499574</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>BV Lâm Đồng</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>11315074780</v>
+      </c>
+      <c r="C39" t="n">
+        <v>10805692943</v>
+      </c>
+      <c r="D39" t="n">
+        <v>9777460328</v>
+      </c>
+      <c r="E39" t="n">
+        <v>14617111861</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>BV Lạng Sơn</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>3806673988</v>
+      </c>
+      <c r="C40" t="n">
+        <v>4836134027</v>
+      </c>
+      <c r="D40" t="n">
+        <v>5085294597</v>
+      </c>
+      <c r="E40" t="n">
+        <v>6209087554</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>BV Mỹ Đình</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>28913622959</v>
+      </c>
+      <c r="C41" t="n">
+        <v>19895748725</v>
+      </c>
+      <c r="D41" t="n">
+        <v>25824643919</v>
+      </c>
+      <c r="E41" t="n">
+        <v>22915105091</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>BV Nam Bình Dương</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>16782380153</v>
+      </c>
+      <c r="C42" t="n">
+        <v>15568500921</v>
+      </c>
+      <c r="D42" t="n">
+        <v>11999355596</v>
+      </c>
+      <c r="E42" t="n">
+        <v>17039773860</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>BV Nam Định</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>4817992620</v>
+      </c>
+      <c r="C43" t="n">
+        <v>6826692057</v>
+      </c>
+      <c r="D43" t="n">
+        <v>9388649883</v>
+      </c>
+      <c r="E43" t="n">
+        <v>9221667209</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>BV Nghệ An</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>29880366714</v>
+      </c>
+      <c r="C44" t="n">
+        <v>35059649255</v>
+      </c>
+      <c r="D44" t="n">
+        <v>37552981125</v>
+      </c>
+      <c r="E44" t="n">
+        <v>55223347983</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>BV Ninh Bình</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>4949334201</v>
+      </c>
+      <c r="C45" t="n">
+        <v>6819145736</v>
+      </c>
+      <c r="D45" t="n">
+        <v>8539127594</v>
+      </c>
+      <c r="E45" t="n">
+        <v>14199929326</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>BV Ninh Thuận</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>6514509428</v>
+      </c>
+      <c r="C46" t="n">
+        <v>7340197781</v>
+      </c>
+      <c r="D46" t="n">
+        <v>9027157961</v>
+      </c>
+      <c r="E46" t="n">
+        <v>8159321264</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>BV Phú Mỹ</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>25927014030</v>
+      </c>
+      <c r="C47" t="n">
+        <v>31027473514</v>
+      </c>
+      <c r="D47" t="n">
+        <v>19543061102</v>
+      </c>
+      <c r="E47" t="n">
+        <v>29440733857</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>BV Phú Quốc</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>2307148907</v>
+      </c>
+      <c r="C48" t="n">
+        <v>3143480330</v>
+      </c>
+      <c r="D48" t="n">
+        <v>3616359475</v>
+      </c>
+      <c r="E48" t="n">
+        <v>6027065156</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>BV Phú Thọ</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>10474041681</v>
+      </c>
+      <c r="C49" t="n">
+        <v>7400968369</v>
+      </c>
+      <c r="D49" t="n">
+        <v>15808417066</v>
+      </c>
+      <c r="E49" t="n">
+        <v>16041482881</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>BV Phú Yên</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>6001220698</v>
+      </c>
+      <c r="C50" t="n">
+        <v>6072129406</v>
+      </c>
+      <c r="D50" t="n">
+        <v>9916779233</v>
+      </c>
+      <c r="E50" t="n">
+        <v>11932175996</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>BV Quảng Bình</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>7763544446</v>
+      </c>
+      <c r="C51" t="n">
+        <v>9556390231</v>
+      </c>
+      <c r="D51" t="n">
+        <v>9655351364</v>
+      </c>
+      <c r="E51" t="n">
+        <v>11340636061</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>BV Quảng Nam</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>15083969818</v>
+      </c>
+      <c r="C52" t="n">
+        <v>17036207012</v>
+      </c>
+      <c r="D52" t="n">
+        <v>21048877988</v>
+      </c>
+      <c r="E52" t="n">
+        <v>25098107314</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>BV Quảng Ngãi</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>6978010604</v>
+      </c>
+      <c r="C53" t="n">
+        <v>7339893831</v>
+      </c>
+      <c r="D53" t="n">
+        <v>8297048712</v>
+      </c>
+      <c r="E53" t="n">
+        <v>9463862174</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>BV Quảng Ninh</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>12481811955</v>
+      </c>
+      <c r="C54" t="n">
+        <v>13414872173</v>
+      </c>
+      <c r="D54" t="n">
+        <v>12737033401</v>
+      </c>
+      <c r="E54" t="n">
+        <v>19298717206</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>BV Quảng Trị</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>9919819591</v>
+      </c>
+      <c r="C55" t="n">
+        <v>10549538572</v>
+      </c>
+      <c r="D55" t="n">
+        <v>10018248512</v>
+      </c>
+      <c r="E55" t="n">
+        <v>17325184586</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>BV Sài Gòn</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>137653679526</v>
+      </c>
+      <c r="C56" t="n">
+        <v>146272797596</v>
+      </c>
+      <c r="D56" t="n">
+        <v>77381834846</v>
+      </c>
+      <c r="E56" t="n">
+        <v>79548826628</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>BV Sóc Trăng</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>6162830285</v>
+      </c>
+      <c r="C57" t="n">
+        <v>7148387094</v>
+      </c>
+      <c r="D57" t="n">
+        <v>8523735726</v>
+      </c>
+      <c r="E57" t="n">
+        <v>7321301077</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>BV Sơn La</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>7376196546</v>
+      </c>
+      <c r="C58" t="n">
+        <v>8300094135</v>
+      </c>
+      <c r="D58" t="n">
+        <v>8088497256</v>
+      </c>
+      <c r="E58" t="n">
+        <v>9995375979</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>BV Sơn Tây</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>13224496942</v>
+      </c>
+      <c r="C59" t="n">
+        <v>15963747610</v>
+      </c>
+      <c r="D59" t="n">
+        <v>23975020089</v>
+      </c>
+      <c r="E59" t="n">
+        <v>32531193806</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>BV Thanh Hóa</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>8707254175</v>
+      </c>
+      <c r="C60" t="n">
+        <v>10752523831</v>
+      </c>
+      <c r="D60" t="n">
+        <v>11677983240</v>
+      </c>
+      <c r="E60" t="n">
+        <v>15146162727</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>BV Thành phố HCM</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>60550799129</v>
+      </c>
+      <c r="C61" t="n">
+        <v>43119724675</v>
+      </c>
+      <c r="D61" t="n">
+        <v>43861789420</v>
+      </c>
+      <c r="E61" t="n">
+        <v>51021500500</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>BV Thái Bình</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>13202876599</v>
+      </c>
+      <c r="C62" t="n">
+        <v>29839517179</v>
+      </c>
+      <c r="D62" t="n">
+        <v>6270820914</v>
+      </c>
+      <c r="E62" t="n">
+        <v>14235360047</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>BV Thái Nguyên</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>9802838868</v>
+      </c>
+      <c r="C63" t="n">
+        <v>10337702301</v>
+      </c>
+      <c r="D63" t="n">
+        <v>19026483839</v>
+      </c>
+      <c r="E63" t="n">
+        <v>14641846440</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>BV Thăng Long</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>25319273655</v>
+      </c>
+      <c r="C64" t="n">
+        <v>22033735424</v>
+      </c>
+      <c r="D64" t="n">
+        <v>29435997445</v>
+      </c>
+      <c r="E64" t="n">
+        <v>31974602442</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>BV Thừa Thiên Huế</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>10464847897</v>
+      </c>
+      <c r="C65" t="n">
+        <v>10658608902</v>
+      </c>
+      <c r="D65" t="n">
+        <v>12537092097</v>
+      </c>
+      <c r="E65" t="n">
+        <v>20244476724</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>BV Tiền Giang</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>6209585313</v>
+      </c>
+      <c r="C66" t="n">
+        <v>5756133242</v>
+      </c>
+      <c r="D66" t="n">
+        <v>36230383145</v>
+      </c>
+      <c r="E66" t="n">
+        <v>7902853487</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>BV Trà Vinh</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>4805927996</v>
+      </c>
+      <c r="C67" t="n">
+        <v>4601290915</v>
+      </c>
+      <c r="D67" t="n">
+        <v>5914090280</v>
+      </c>
+      <c r="E67" t="n">
+        <v>8300348130</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>BV Tràng An</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>15410418570</v>
+      </c>
+      <c r="C68" t="n">
+        <v>19110506849</v>
+      </c>
+      <c r="D68" t="n">
+        <v>20211788652</v>
+      </c>
+      <c r="E68" t="n">
+        <v>25233173814</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>BV Tuyên Quang</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>4559487348</v>
+      </c>
+      <c r="C69" t="n">
+        <v>4839722740</v>
+      </c>
+      <c r="D69" t="n">
+        <v>5474315672</v>
+      </c>
+      <c r="E69" t="n">
+        <v>6413159336</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>BV Tây Ninh</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>5457968705</v>
+      </c>
+      <c r="C70" t="n">
+        <v>20165458513</v>
+      </c>
+      <c r="D70" t="n">
+        <v>11679865762</v>
+      </c>
+      <c r="E70" t="n">
+        <v>17863919258</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>BV Vĩnh Long</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>7539677151</v>
+      </c>
+      <c r="C71" t="n">
+        <v>7385288620</v>
+      </c>
+      <c r="D71" t="n">
+        <v>23841315898</v>
+      </c>
+      <c r="E71" t="n">
+        <v>14595134471</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>BV Vĩnh Phúc</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>8115397059</v>
+      </c>
+      <c r="C72" t="n">
+        <v>9891104441</v>
+      </c>
+      <c r="D72" t="n">
+        <v>8973711908</v>
+      </c>
+      <c r="E72" t="n">
+        <v>10801132649</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>BV Yên Bái</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>3259538472</v>
+      </c>
+      <c r="C73" t="n">
+        <v>3610078629</v>
+      </c>
+      <c r="D73" t="n">
+        <v>4341550885</v>
+      </c>
+      <c r="E73" t="n">
+        <v>8492418016</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>BV Điện Biên</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>6413387929</v>
+      </c>
+      <c r="C74" t="n">
+        <v>5270875966</v>
+      </c>
+      <c r="D74" t="n">
+        <v>7700250744</v>
+      </c>
+      <c r="E74" t="n">
+        <v>11897663707</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>BV Đà Nẵng</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>47975717233</v>
+      </c>
+      <c r="C75" t="n">
+        <v>38852839962</v>
+      </c>
+      <c r="D75" t="n">
+        <v>37992096820</v>
+      </c>
+      <c r="E75" t="n">
+        <v>51159912583</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>BV Đình Vũ</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>4074932511</v>
+      </c>
+      <c r="C76" t="n">
+        <v>9261134775</v>
+      </c>
+      <c r="D76" t="n">
+        <v>5670103369</v>
+      </c>
+      <c r="E76" t="n">
+        <v>7456649552</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>BV Đông Bắc</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>5565158236</v>
+      </c>
+      <c r="C77" t="n">
+        <v>5561976751</v>
+      </c>
+      <c r="D77" t="n">
+        <v>4277687902</v>
+      </c>
+      <c r="E77" t="n">
+        <v>4512537003</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>BV Đông Đô</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>41301631580</v>
+      </c>
+      <c r="C78" t="n">
+        <v>109903595412</v>
+      </c>
+      <c r="D78" t="n">
+        <v>69252704144</v>
+      </c>
+      <c r="E78" t="n">
+        <v>77959039223</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>BV Đồng Nai</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>7661529495</v>
+      </c>
+      <c r="C79" t="n">
+        <v>7949774820</v>
+      </c>
+      <c r="D79" t="n">
+        <v>20853719775</v>
+      </c>
+      <c r="E79" t="n">
+        <v>33002600237</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>BV Đồng Tháp</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>13054880587</v>
+      </c>
+      <c r="C80" t="n">
+        <v>8745841217</v>
+      </c>
+      <c r="D80" t="n">
+        <v>30523450752</v>
+      </c>
+      <c r="E80" t="n">
+        <v>40752735867</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Trụ sở chính</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>581181000896</v>
+      </c>
+      <c r="C81" t="n">
+        <v>285839516311</v>
+      </c>
+      <c r="D81" t="n">
+        <v>382479650841</v>
+      </c>
+      <c r="E81" t="n">
+        <v>237631151398</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>